<commit_message>
Updated  Projects Field information in excel files
</commit_message>
<xml_diff>
--- a/python/table_metadata.xlsx
+++ b/python/table_metadata.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9840" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="10440" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="764" uniqueCount="324">
   <si>
     <t>TableName</t>
   </si>
@@ -763,6 +763,30 @@
   </si>
   <si>
     <t>User who created — INTEGER FK. JOIN AbpUsers ON CreatorUserId=Id. NEVER filter by username directly.</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "Projects"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "WorkOrders"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "AbpUsers"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "AbpOrganizationUnits"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "Offices"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "AbpRoles"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "Clients"."IsDeleted" = false — never bare "IsDeleted"</t>
+  </si>
+  <si>
+    <t>Soft delete. Always write "Phases"."IsDeleted" = false — never bare "IsDeleted"</t>
   </si>
   <si>
     <t>FromTable</t>
@@ -1624,7 +1648,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1644,6 +1668,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="distributed"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2011,13 +2038,13 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2307,7 +2334,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D114"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -3374,7 +3401,7 @@
       <c r="C76" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D76" s="10" t="s">
+      <c r="D76" s="11" t="s">
         <v>91</v>
       </c>
     </row>
@@ -3733,6 +3760,94 @@
       </c>
       <c r="D106" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="107" ht="28.8" spans="1:4">
+      <c r="A107" t="s">
+        <v>68</v>
+      </c>
+      <c r="B107" t="s">
+        <v>120</v>
+      </c>
+      <c r="C107" s="9" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="108" ht="28.8" spans="1:4">
+      <c r="A108" t="s">
+        <v>4</v>
+      </c>
+      <c r="B108" t="s">
+        <v>120</v>
+      </c>
+      <c r="C108" s="9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="109" ht="28.8" spans="1:4">
+      <c r="A109" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" t="s">
+        <v>120</v>
+      </c>
+      <c r="C109" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="110" ht="28.8" spans="1:4">
+      <c r="A110" t="s">
+        <v>59</v>
+      </c>
+      <c r="B110" t="s">
+        <v>120</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="111" ht="28.8" spans="1:4">
+      <c r="A111" t="s">
+        <v>8</v>
+      </c>
+      <c r="B111" t="s">
+        <v>120</v>
+      </c>
+      <c r="C111" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="112" ht="28.8" spans="1:4">
+      <c r="A112" t="s">
+        <v>16</v>
+      </c>
+      <c r="B112" t="s">
+        <v>120</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3">
+      <c r="A113" t="s">
+        <v>40</v>
+      </c>
+      <c r="B113" t="s">
+        <v>120</v>
+      </c>
+      <c r="C113" s="9" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="114" ht="28.8" spans="1:3">
+      <c r="A114" t="s">
+        <v>50</v>
+      </c>
+      <c r="B114" t="s">
+        <v>120</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -3754,19 +3869,19 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:5">
@@ -3783,7 +3898,7 @@
         <v>74</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" spans="1:5">
@@ -3800,7 +3915,7 @@
         <v>74</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:5">
@@ -3817,7 +3932,7 @@
         <v>74</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:5">
@@ -3834,7 +3949,7 @@
         <v>74</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:5">
@@ -3851,7 +3966,7 @@
         <v>74</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:5">
@@ -3868,7 +3983,7 @@
         <v>74</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:5">
@@ -3885,7 +4000,7 @@
         <v>74</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:5">
@@ -3893,16 +4008,16 @@
         <v>4</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:5">
@@ -3913,13 +4028,13 @@
         <v>102</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:5">
@@ -3930,13 +4045,13 @@
         <v>105</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:5">
@@ -3953,7 +4068,7 @@
         <v>74</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:5">
@@ -3970,7 +4085,7 @@
         <v>74</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:5">
@@ -3987,7 +4102,7 @@
         <v>74</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:5">
@@ -4004,7 +4119,7 @@
         <v>74</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:5">
@@ -4021,7 +4136,7 @@
         <v>74</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:5">
@@ -4038,7 +4153,7 @@
         <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:5">
@@ -4055,7 +4170,7 @@
         <v>74</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:5">
@@ -4072,7 +4187,7 @@
         <v>74</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:5">
@@ -4089,7 +4204,7 @@
         <v>74</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:5">
@@ -4106,7 +4221,7 @@
         <v>74</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:5">
@@ -4123,7 +4238,7 @@
         <v>74</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:5">
@@ -4140,7 +4255,7 @@
         <v>74</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" spans="1:5">
@@ -4157,7 +4272,7 @@
         <v>74</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" spans="1:5">
@@ -4174,7 +4289,7 @@
         <v>74</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1" spans="1:5">
@@ -4182,7 +4297,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>44</v>
@@ -4191,7 +4306,7 @@
         <v>74</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1" spans="1:5">
@@ -4202,13 +4317,13 @@
         <v>199</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>74</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1" spans="1:5">
@@ -4225,7 +4340,7 @@
         <v>74</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:5">
@@ -4242,7 +4357,7 @@
         <v>74</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:5">
@@ -4259,7 +4374,7 @@
         <v>74</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:5">
@@ -4276,7 +4391,7 @@
         <v>74</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1" spans="1:5">
@@ -4287,13 +4402,13 @@
         <v>155</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>74</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4310,7 +4425,7 @@
         <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4321,13 +4436,13 @@
         <v>99</v>
       </c>
       <c r="C34" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="D34" t="s">
         <v>74</v>
       </c>
       <c r="E34" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -4344,7 +4459,7 @@
         <v>74</v>
       </c>
       <c r="E35" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -4361,7 +4476,7 @@
         <v>74</v>
       </c>
       <c r="E36" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -4378,7 +4493,7 @@
         <v>74</v>
       </c>
       <c r="E37" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -4395,7 +4510,7 @@
         <v>74</v>
       </c>
       <c r="E38" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -4412,7 +4527,7 @@
         <v>74</v>
       </c>
       <c r="E39" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>
@@ -4437,10 +4552,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -4448,10 +4563,10 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="C2" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -4459,10 +4574,10 @@
         <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C3" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -4470,10 +4585,10 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C4" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -4481,10 +4596,10 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="C5" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -4492,10 +4607,10 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="C6" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -4503,10 +4618,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="C7" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -4514,10 +4629,10 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C8" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -4525,10 +4640,10 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="C9" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -4536,10 +4651,10 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="C10" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -4547,10 +4662,10 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
+        <v>310</v>
+      </c>
+      <c r="C11" t="s">
         <v>302</v>
-      </c>
-      <c r="C11" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -4558,10 +4673,10 @@
         <v>47</v>
       </c>
       <c r="B12" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="C12" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -4569,10 +4684,10 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="C13" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -4580,10 +4695,10 @@
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C14" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -4591,10 +4706,10 @@
         <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="C15" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -4602,32 +4717,32 @@
         <v>37</v>
       </c>
       <c r="B16" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C16" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="B17" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C17" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="B18" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="C18" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -4635,10 +4750,10 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C19" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -4646,10 +4761,10 @@
         <v>65</v>
       </c>
       <c r="B20" t="s">
+        <v>323</v>
+      </c>
+      <c r="C20" t="s">
         <v>315</v>
-      </c>
-      <c r="C20" t="s">
-        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>